<commit_message>
[ENH] Modified instructions, sf module parameters and added end of experiment routine
</commit_message>
<xml_diff>
--- a/src/instructions/color_staircase_instructions.xlsx
+++ b/src/instructions/color_staircase_instructions.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27928"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28925"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\akoun\Desktop\Biocruces\siburmuin\src\begiBrainDemo\instructions\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\akoun\Desktop\Biocruces\begibraintool\src\instructions\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6C6935D3-CC33-48DD-8D4B-914304DA3A0C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9D4B8442-02E4-4567-BF32-1700E3BCF540}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="2175" yWindow="2175" windowWidth="16200" windowHeight="9308" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="12975" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -116,14 +116,20 @@
     <t>instruction_5</t>
   </si>
   <si>
-    <t>Pulsa la barra espaciadora cuando quieras empezar la prueba</t>
-  </si>
-  <si>
     <t>COLOR/SATURATION  THRESHOLD STAIRCASE TEST</t>
   </si>
   <si>
+    <t>Si no puedes ver las líneas pulsa el botón central. Si ves que las líneas van de izquierda a derecha pulsa el botón derecho.</t>
+  </si>
+  <si>
+    <t>Si ves que las líneas van de derecha a izquierda pulsa el botón izquierdo.</t>
+  </si>
+  <si>
+    <t>Si has entendido las instrucciones, pulsa el botón central para empezar la prueba. Pregunta si tienes dudas.</t>
+  </si>
+  <si>
     <r>
-      <t>Observa la pantalla</t>
+      <t>Muy bien. Ahora repetiremos la prueba modificando los colores del parche. Observa la pantalla</t>
     </r>
     <r>
       <rPr>
@@ -133,36 +139,7 @@
         <family val="2"/>
         <scheme val="minor"/>
       </rPr>
-      <t>: Aparecerá un patrón de líneas con diferentes colores.</t>
-    </r>
-  </si>
-  <si>
-    <t>Si puedes diferenciar los colores, pulsa la tecla S.</t>
-  </si>
-  <si>
-    <r>
-      <t xml:space="preserve">Si ves un color uniforme, pulsa la tecla </t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>N</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>.</t>
+      <t>: Aparecerá un patrón de líneas</t>
     </r>
   </si>
 </sst>
@@ -594,19 +571,19 @@
     </row>
     <row r="2" spans="1:6" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A2" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="B2" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="C2" t="s">
         <v>7</v>
       </c>
-      <c r="B2" s="3" t="s">
+      <c r="D2" t="s">
         <v>8</v>
       </c>
-      <c r="C2" s="3" t="s">
+      <c r="E2" t="s">
         <v>9</v>
-      </c>
-      <c r="D2" t="s">
-        <v>10</v>
-      </c>
-      <c r="F2" t="s">
-        <v>6</v>
       </c>
     </row>
   </sheetData>
@@ -622,6 +599,21 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement/>
+</p:properties>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100B9F5CAB0486A994CA2C3B13E059EF2AE" ma:contentTypeVersion="0" ma:contentTypeDescription="Een nieuw document maken." ma:contentTypeScope="" ma:versionID="8645ec4a60d0c8c7009d2d6675847a91">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="636d7205651659ec4fcda0bcbde9384b">
     <xsd:element name="properties">
@@ -735,22 +727,30 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement/>
-</p:properties>
-</file>
-
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{B3725960-8A89-4E70-9C40-340E0EDB6403}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{3744155D-8FAB-4E67-B5E0-C7FDBFB3715D}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{EFF1C174-6AC6-4774-A736-3226A12360E4}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -764,27 +764,4 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{3744155D-8FAB-4E67-B5E0-C7FDBFB3715D}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{B3725960-8A89-4E70-9C40-340E0EDB6403}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
 </file>
</xml_diff>